<commit_message>
#16 Quantity Per Board Column Name updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/FLST_PCBWay BOM.xlsx
+++ b/Deliverables/BOM/FLST_PCBWay BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\flst\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70144D4-DC3E-41AC-8A95-0A79B9A9BC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614B6B70-2A9C-49DB-A515-7DBE31ABA526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>LCSC/Part No</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
     <t>LCSC/MOQ/5 Boards</t>
   </si>
   <si>
@@ -504,6 +501,9 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>Quantity (Per Board)</t>
   </si>
 </sst>
 </file>
@@ -1048,6 +1048,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1080,9 +1083,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1106,11 +1106,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>57151</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>28576</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="1114424"/>
+    <xdr:ext cx="2686049" cy="1114424"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1">
@@ -1137,8 +1137,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12068176" y="638176"/>
-          <a:ext cx="2000250" cy="1114424"/>
+          <a:off x="10934700" y="638176"/>
+          <a:ext cx="2686049" cy="1114424"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1424,6 +1424,7 @@
     <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1436,18 +1437,18 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
     </row>
     <row r="2" spans="1:11" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="9"/>
@@ -1460,52 +1461,52 @@
       <c r="A3" s="2"/>
       <c r="B3" s="10"/>
       <c r="C3" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D3" s="36"/>
       <c r="E3" s="37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F3" s="36"/>
       <c r="G3" s="38"/>
       <c r="H3" s="38"/>
       <c r="I3" s="38"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="54"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="55"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="10"/>
       <c r="C4" s="36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D4" s="36"/>
       <c r="E4" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="55"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="56"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="10"/>
       <c r="C5" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" s="36"/>
       <c r="E5" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="55"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="56"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -1517,8 +1518,8 @@
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
-      <c r="J6" s="58"/>
-      <c r="K6" s="55"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="56"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -1530,8 +1531,8 @@
       <c r="G7" s="40"/>
       <c r="H7" s="40"/>
       <c r="I7" s="40"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="55"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="56"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -1543,13 +1544,13 @@
       <c r="G8" s="40"/>
       <c r="H8" s="40"/>
       <c r="I8" s="40"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="56"/>
+      <c r="J8" s="60"/>
+      <c r="K8" s="57"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>0</v>
@@ -1564,19 +1565,19 @@
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="K9" s="24" t="s">
         <v>5</v>
-      </c>
-      <c r="K9" s="24" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1586,25 +1587,25 @@
         <v>1</v>
       </c>
       <c r="C10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="E10" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="F10" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="G10" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="H10" s="25" t="s">
+      <c r="I10" s="26" t="s">
         <v>11</v>
-      </c>
-      <c r="I10" s="26" t="s">
-        <v>12</v>
       </c>
       <c r="J10" s="25">
         <v>1</v>
@@ -1620,25 +1621,25 @@
         <v>2</v>
       </c>
       <c r="C11" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="E11" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="F11" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="G11" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="H11" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="H11" s="27" t="s">
+      <c r="I11" s="28" t="s">
         <v>17</v>
-      </c>
-      <c r="I11" s="28" t="s">
-        <v>18</v>
       </c>
       <c r="J11" s="27">
         <v>1</v>
@@ -1654,25 +1655,25 @@
         <v>3</v>
       </c>
       <c r="C12" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="E12" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="F12" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="G12" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="H12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H12" s="25" t="s">
+      <c r="I12" s="26" t="s">
         <v>23</v>
-      </c>
-      <c r="I12" s="26" t="s">
-        <v>24</v>
       </c>
       <c r="J12" s="25">
         <v>1</v>
@@ -1688,25 +1689,25 @@
         <v>4</v>
       </c>
       <c r="C13" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="E13" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="28" t="s">
+      <c r="G13" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="H13" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="H13" s="27" t="s">
+      <c r="I13" s="28" t="s">
         <v>28</v>
-      </c>
-      <c r="I13" s="28" t="s">
-        <v>29</v>
       </c>
       <c r="J13" s="27">
         <v>2</v>
@@ -1722,25 +1723,25 @@
         <v>5</v>
       </c>
       <c r="C14" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="E14" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="26" t="s">
+      <c r="G14" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="H14" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H14" s="25" t="s">
+      <c r="I14" s="26" t="s">
         <v>33</v>
-      </c>
-      <c r="I14" s="26" t="s">
-        <v>34</v>
       </c>
       <c r="J14" s="25">
         <v>1</v>
@@ -1756,25 +1757,25 @@
         <v>6</v>
       </c>
       <c r="C15" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="E15" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="F15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="28" t="s">
+      <c r="G15" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="H15" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="G15" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="H15" s="27" t="s">
+      <c r="I15" s="28" t="s">
         <v>39</v>
-      </c>
-      <c r="I15" s="28" t="s">
-        <v>40</v>
       </c>
       <c r="J15" s="27">
         <v>1</v>
@@ -1790,25 +1791,25 @@
         <v>7</v>
       </c>
       <c r="C16" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="E16" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="F16" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="G16" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="H16" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="25" t="s">
-        <v>138</v>
-      </c>
-      <c r="H16" s="25" t="s">
+      <c r="I16" s="26" t="s">
         <v>45</v>
-      </c>
-      <c r="I16" s="26" t="s">
-        <v>46</v>
       </c>
       <c r="J16" s="25">
         <v>1</v>
@@ -1824,25 +1825,25 @@
         <v>8</v>
       </c>
       <c r="C17" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="E17" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="28" t="s">
+      <c r="G17" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="H17" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="G17" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="H17" s="27" t="s">
+      <c r="I17" s="28" t="s">
         <v>50</v>
-      </c>
-      <c r="I17" s="28" t="s">
-        <v>51</v>
       </c>
       <c r="J17" s="27">
         <v>1</v>
@@ -1858,25 +1859,25 @@
         <v>9</v>
       </c>
       <c r="C18" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="E18" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="E18" s="25" t="s">
+      <c r="F18" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="G18" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="H18" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="H18" s="25" t="s">
-        <v>56</v>
-      </c>
       <c r="I18" s="26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J18" s="25">
         <v>1</v>
@@ -1892,25 +1893,25 @@
         <v>10</v>
       </c>
       <c r="C19" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="E19" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="F19" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="F19" s="60" t="s">
+      <c r="G19" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="H19" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="G19" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="H19" s="27" t="s">
-        <v>61</v>
-      </c>
       <c r="I19" s="28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J19" s="27">
         <v>10</v>
@@ -1926,22 +1927,22 @@
         <v>11</v>
       </c>
       <c r="C20" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="E20" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="E20" s="25" t="s">
+      <c r="F20" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="F20" s="26" t="s">
+      <c r="G20" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="H20" s="25" t="s">
         <v>65</v>
-      </c>
-      <c r="G20" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="H20" s="25" t="s">
-        <v>66</v>
       </c>
       <c r="I20" s="26"/>
       <c r="J20" s="25">
@@ -1958,25 +1959,25 @@
         <v>12</v>
       </c>
       <c r="C21" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="E21" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="F21" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="G21" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="H21" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="G21" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="H21" s="27" t="s">
+      <c r="I21" s="28" t="s">
         <v>71</v>
-      </c>
-      <c r="I21" s="28" t="s">
-        <v>72</v>
       </c>
       <c r="J21" s="27">
         <v>1</v>
@@ -1992,25 +1993,25 @@
         <v>13</v>
       </c>
       <c r="C22" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="E22" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="E22" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="F22" s="26" t="s">
+      <c r="G22" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="H22" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="G22" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H22" s="25" t="s">
+      <c r="I22" s="26" t="s">
         <v>76</v>
-      </c>
-      <c r="I22" s="26" t="s">
-        <v>77</v>
       </c>
       <c r="J22" s="25">
         <v>1</v>
@@ -2026,25 +2027,25 @@
         <v>14</v>
       </c>
       <c r="C23" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="E23" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="F23" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="G23" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="H23" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="G23" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="H23" s="27" t="s">
+      <c r="I23" s="28" t="s">
         <v>82</v>
-      </c>
-      <c r="I23" s="28" t="s">
-        <v>83</v>
       </c>
       <c r="J23" s="27">
         <v>4</v>
@@ -2060,25 +2061,25 @@
         <v>15</v>
       </c>
       <c r="C24" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D24" s="25" t="s">
+      <c r="E24" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="F24" s="26" t="s">
+      <c r="G24" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="H24" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="G24" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="H24" s="25" t="s">
+      <c r="I24" s="26" t="s">
         <v>87</v>
-      </c>
-      <c r="I24" s="26" t="s">
-        <v>88</v>
       </c>
       <c r="J24" s="25">
         <v>5</v>
@@ -2094,25 +2095,25 @@
         <v>16</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D25" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="E25" s="27" t="s">
+      <c r="F25" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="G25" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="H25" s="27" t="s">
         <v>146</v>
       </c>
-      <c r="G25" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="H25" s="27" t="s">
+      <c r="I25" s="28" t="s">
         <v>147</v>
-      </c>
-      <c r="I25" s="28" t="s">
-        <v>148</v>
       </c>
       <c r="J25" s="27">
         <v>5</v>
@@ -2128,25 +2129,25 @@
         <v>17</v>
       </c>
       <c r="C26" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="E26" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="E26" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="F26" s="26" t="s">
+      <c r="G26" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="G26" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H26" s="25" t="s">
+      <c r="I26" s="26" t="s">
         <v>93</v>
-      </c>
-      <c r="I26" s="26" t="s">
-        <v>94</v>
       </c>
       <c r="J26" s="25">
         <v>1</v>
@@ -2162,25 +2163,25 @@
         <v>18</v>
       </c>
       <c r="C27" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="27" t="s">
+      <c r="E27" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="E27" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="F27" s="28" t="s">
+      <c r="G27" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="H27" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G27" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="H27" s="27" t="s">
+      <c r="I27" s="28" t="s">
         <v>98</v>
-      </c>
-      <c r="I27" s="28" t="s">
-        <v>99</v>
       </c>
       <c r="J27" s="27">
         <v>1</v>
@@ -2196,25 +2197,25 @@
         <v>19</v>
       </c>
       <c r="C28" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="D28" s="25" t="s">
+      <c r="E28" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="E28" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="F28" s="26" t="s">
+      <c r="G28" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="H28" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="G28" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="H28" s="25" t="s">
-        <v>103</v>
-      </c>
       <c r="I28" s="26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J28" s="25">
         <v>1</v>
@@ -2230,25 +2231,25 @@
         <v>20</v>
       </c>
       <c r="C29" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="D29" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D29" s="27" t="s">
+      <c r="E29" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="F29" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="F29" s="28" t="s">
+      <c r="G29" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="H29" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="G29" s="27" t="s">
-        <v>151</v>
-      </c>
-      <c r="H29" s="27" t="s">
-        <v>108</v>
-      </c>
       <c r="I29" s="28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J29" s="27">
         <v>1</v>
@@ -2264,25 +2265,25 @@
         <v>21</v>
       </c>
       <c r="C30" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="E30" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="E30" s="25" t="s">
+      <c r="F30" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="F30" s="26" t="s">
+      <c r="G30" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="H30" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="G30" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="H30" s="25" t="s">
-        <v>113</v>
-      </c>
       <c r="I30" s="26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J30" s="25">
         <v>1</v>
@@ -2298,25 +2299,25 @@
         <v>22</v>
       </c>
       <c r="C31" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="D31" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="D31" s="27" t="s">
+      <c r="E31" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="E31" s="27" t="s">
+      <c r="F31" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="28" t="s">
+      <c r="G31" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="H31" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="H31" s="27" t="s">
-        <v>118</v>
-      </c>
       <c r="I31" s="28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J31" s="27">
         <v>1</v>
@@ -2332,25 +2333,25 @@
         <v>23</v>
       </c>
       <c r="C32" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="E32" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="E32" s="29" t="s">
+      <c r="F32" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="F32" s="30" t="s">
+      <c r="G32" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="H32" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="G32" s="29" t="s">
-        <v>154</v>
-      </c>
-      <c r="H32" s="29" t="s">
-        <v>123</v>
-      </c>
       <c r="I32" s="30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J32" s="29">
         <v>1</v>
@@ -2363,31 +2364,31 @@
       <c r="A33" s="2"/>
       <c r="B33" s="31"/>
       <c r="C33" s="46" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D33" s="47"/>
       <c r="E33" s="48"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="50"/>
+      <c r="F33" s="50"/>
+      <c r="G33" s="50"/>
+      <c r="H33" s="50"/>
+      <c r="I33" s="50"/>
+      <c r="J33" s="50"/>
+      <c r="K33" s="51"/>
     </row>
     <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="32"/>
       <c r="C34" s="33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D34" s="34"/>
       <c r="E34" s="34"/>
-      <c r="F34" s="51"/>
-      <c r="G34" s="51"/>
-      <c r="H34" s="51"/>
-      <c r="I34" s="51"/>
-      <c r="J34" s="51"/>
-      <c r="K34" s="52"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="52"/>
+      <c r="H34" s="52"/>
+      <c r="I34" s="52"/>
+      <c r="J34" s="52"/>
+      <c r="K34" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>